<commit_message>
2×2 raffiné : dédoublonnage physique, Cornwall + Fallowfield, dispersion par sillon
Paires physiques uniques (double-CN n=20 → 12, pseudo-réplication corrigée).
Cornwall (km 112,8 projeté, écart 2 m) coupe le géant Dorval-Brockville ;
Fallowfield (km 15,4) isole l'approche d'Ottawa (158 % exclue) et libère
Fallowfield-Smiths Falls (51 %, simple-VIA pur). Nouvelle colonne dispersion
inter-sillons : IQR médian double-CN 6,4 % / simple-VIA 10,0 % / simple-CN
21,4 % = deuxième signature du régime. Médianes : 38,5 / 42,0 / 65,2.

Co-Authored-By: Claude Fable 5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01UAqHM1ry5Ckx2YL5NLcNpH
</commit_message>
<xml_diff>
--- a/livrables/marges_2x2_synthese.xlsx
+++ b/livrables/marges_2x2_synthese.xlsx
@@ -10,7 +10,7 @@
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="marges_2x2_synthese" sheetId="1" state="visible" r:id="rId1"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'marges_2x2_synthese'!$A$1:$G$4</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'marges_2x2_synthese'!$A$1:$H$4</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
@@ -427,7 +427,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:G4"/>
+  <dimension ref="A1:H4"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="12" customWidth="1" min="1" max="1"/>
@@ -437,6 +437,7 @@
     <col width="8" customWidth="1" min="5" max="5"/>
     <col width="9" customWidth="1" min="6" max="6"/>
     <col width="9" customWidth="1" min="7" max="7"/>
+    <col width="18" customWidth="1" min="8" max="8"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -475,6 +476,11 @@
           <t>maximum</t>
         </is>
       </c>
+      <c r="H1" s="1" t="inlineStr">
+        <is>
+          <t>disp_iqr_pct_med</t>
+        </is>
+      </c>
     </row>
     <row r="2">
       <c r="A2" t="inlineStr">
@@ -483,22 +489,25 @@
         </is>
       </c>
       <c r="B2" t="n">
-        <v>20</v>
+        <v>12</v>
       </c>
       <c r="C2" t="n">
-        <v>42.2</v>
+        <v>38.5</v>
       </c>
       <c r="D2" t="n">
-        <v>36.2</v>
+        <v>34.6</v>
       </c>
       <c r="E2" t="n">
-        <v>49.6</v>
+        <v>45.7</v>
       </c>
       <c r="F2" t="n">
-        <v>32.4</v>
+        <v>32.3</v>
       </c>
       <c r="G2" t="n">
-        <v>72.7</v>
+        <v>69.8</v>
+      </c>
+      <c r="H2" t="n">
+        <v>6.4</v>
       </c>
     </row>
     <row r="3">
@@ -525,6 +534,9 @@
       <c r="G3" t="n">
         <v>69.59999999999999</v>
       </c>
+      <c r="H3" t="n">
+        <v>21.4</v>
+      </c>
     </row>
     <row r="4">
       <c r="A4" t="inlineStr">
@@ -542,17 +554,20 @@
         <v>33.2</v>
       </c>
       <c r="E4" t="n">
-        <v>62.5</v>
+        <v>51.4</v>
       </c>
       <c r="F4" t="n">
         <v>24</v>
       </c>
       <c r="G4" t="n">
-        <v>91.40000000000001</v>
+        <v>62.5</v>
+      </c>
+      <c r="H4" t="n">
+        <v>10</v>
       </c>
     </row>
   </sheetData>
-  <autoFilter ref="A1:G4"/>
+  <autoFilter ref="A1:H4"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
2×2 : frontière Metrolinx (Pickering Jct) appliquée, Oshawa-Guildwood hors 2×2
Kingston Union-Pickering = Metrolinx depuis 2011 (29,9 km) ; les paires
chevauchant une frontière de propriétaire sont exclues de la synthèse.
Double-CN épuré : n=11, médiane 36,8 %, dispersion 5,0 %. Lectures :
doublement ≈ 28 pts ; régime : voie simple = +5 pts chez VIA vs +28 chez CN.

Co-Authored-By: Claude Fable 5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01UAqHM1ry5Ckx2YL5NLcNpH
</commit_message>
<xml_diff>
--- a/livrables/marges_2x2_synthese.xlsx
+++ b/livrables/marges_2x2_synthese.xlsx
@@ -489,16 +489,16 @@
         </is>
       </c>
       <c r="B2" t="n">
-        <v>12</v>
+        <v>11</v>
       </c>
       <c r="C2" t="n">
-        <v>38.5</v>
+        <v>36.8</v>
       </c>
       <c r="D2" t="n">
-        <v>34.6</v>
+        <v>34.2</v>
       </c>
       <c r="E2" t="n">
-        <v>45.7</v>
+        <v>44.3</v>
       </c>
       <c r="F2" t="n">
         <v>32.3</v>
@@ -507,7 +507,7 @@
         <v>69.8</v>
       </c>
       <c r="H2" t="n">
-        <v>6.4</v>
+        <v>5</v>
       </c>
     </row>
     <row r="3">

</xml_diff>